<commit_message>
lux tenebris rooster update
</commit_message>
<xml_diff>
--- a/file/history_updated.xlsx
+++ b/file/history_updated.xlsx
@@ -1938,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1968,59 +1968,59 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1783532394458</v>
+        <v>1785396043745</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>FA SIGNING</v>
+        <v>PROMOTED</v>
       </c>
       <c r="D2" t="str">
-        <v>diskyb0b</v>
+        <v>boltz</v>
       </c>
       <c r="E2" t="str">
-        <v>Free Agency</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="F2" t="str">
-        <v>Kappa Bar</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2" t="str">
-        <v>joined as Starter</v>
+        <v>promoted to starter</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>1783532378345</v>
+        <v>1785396042996</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="str">
-        <v>TRANSFER</v>
+        <v>BENCHED</v>
       </c>
       <c r="D3" t="str">
-        <v>Gizmy</v>
+        <v>fer</v>
       </c>
       <c r="E3" t="str">
-        <v>Kappa Bar</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="F3" t="str">
-        <v>Iluminar</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>moved to bench</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1783532335269</v>
+        <v>1785396011356</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -2029,76 +2029,76 @@
         <v>FA SIGNING</v>
       </c>
       <c r="D4" t="str">
-        <v>hades</v>
+        <v>boltz</v>
       </c>
       <c r="E4" t="str">
         <v>Free Agency</v>
       </c>
       <c r="F4" t="str">
-        <v>Mythic</v>
+        <v>Lux Tenebris</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4" t="str">
-        <v>joined as Starter</v>
+        <v>joined as Bench</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>1783532286477</v>
+        <v>1783532394458</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="str">
-        <v>TRANSFER</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D5" t="str">
-        <v>fl0m</v>
+        <v>diskyb0b</v>
       </c>
       <c r="E5" t="str">
-        <v>Mythic</v>
+        <v>Free Agency</v>
       </c>
       <c r="F5" t="str">
-        <v>Iluminar</v>
+        <v>Kappa Bar</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>joined as Starter</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>1783531772696</v>
+        <v>1783532378345</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="str">
-        <v>FA SIGNING</v>
+        <v>TRANSFER</v>
       </c>
       <c r="D6" t="str">
-        <v>taco</v>
+        <v>Gizmy</v>
       </c>
       <c r="E6" t="str">
-        <v>Free Agency</v>
+        <v>Kappa Bar</v>
       </c>
       <c r="F6" t="str">
-        <v>Lux Tenebris</v>
+        <v>Iluminar</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6" t="str">
-        <v>joined as Starter</v>
+        <v>CLAUSE DEAL · joined as Starter</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>1783531758984</v>
+        <v>1783532335269</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -2107,13 +2107,13 @@
         <v>FA SIGNING</v>
       </c>
       <c r="D7" t="str">
-        <v>fer</v>
+        <v>hades</v>
       </c>
       <c r="E7" t="str">
         <v>Free Agency</v>
       </c>
       <c r="F7" t="str">
-        <v>Lux Tenebris</v>
+        <v>Mythic</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -2124,85 +2124,85 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>1783531616692</v>
+        <v>1783532286477</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="str">
-        <v>FA SIGNING</v>
+        <v>TRANSFER</v>
       </c>
       <c r="D8" t="str">
-        <v>kyourezz</v>
+        <v>fl0m</v>
       </c>
       <c r="E8" t="str">
-        <v>Free Agency</v>
+        <v>Mythic</v>
       </c>
       <c r="F8" t="str">
-        <v>Lux Tenebris</v>
+        <v>Iluminar</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8" t="str">
-        <v>joined as Starter</v>
+        <v>CLAUSE DEAL · joined as Starter</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>1783531586211</v>
+        <v>1783531772696</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="str">
-        <v>TRANSFER</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D9" t="str">
-        <v>heroghoxxt</v>
+        <v>taco</v>
       </c>
       <c r="E9" t="str">
-        <v>Iluminar</v>
+        <v>Free Agency</v>
       </c>
       <c r="F9" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G9">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="H9" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>joined as Starter</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>1783531583393</v>
+        <v>1783531758984</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="str">
-        <v>TRANSFER</v>
+        <v>FA SIGNING</v>
       </c>
       <c r="D10" t="str">
-        <v>kilzys</v>
+        <v>fer</v>
       </c>
       <c r="E10" t="str">
-        <v>Iluminar</v>
+        <v>Free Agency</v>
       </c>
       <c r="F10" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G10">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="H10" t="str">
-        <v>CLAUSE DEAL · joined as Starter</v>
+        <v>joined as Starter</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>1783473413103</v>
+        <v>1783531616692</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -2211,7 +2211,7 @@
         <v>FA SIGNING</v>
       </c>
       <c r="D11" t="str">
-        <v>taco</v>
+        <v>kyourezz</v>
       </c>
       <c r="E11" t="str">
         <v>Free Agency</v>
@@ -2228,43 +2228,168 @@
     </row>
     <row r="12">
       <c r="A12">
-        <v>1783473388452</v>
+        <v>1783531586211</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="str">
-        <v>FA SIGNING</v>
+        <v>TRANSFER</v>
       </c>
       <c r="D12" t="str">
-        <v>fer</v>
+        <v>heroghoxxt</v>
       </c>
       <c r="E12" t="str">
-        <v>Free Agency</v>
+        <v>Iluminar</v>
       </c>
       <c r="F12" t="str">
         <v>Lux Tenebris</v>
       </c>
       <c r="G12">
+        <v>40000</v>
+      </c>
+      <c r="H12" t="str">
+        <v>CLAUSE DEAL · joined as Starter</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>1783531583393</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="str">
+        <v>TRANSFER</v>
+      </c>
+      <c r="D13" t="str">
+        <v>kilzys</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Iluminar</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="G13">
+        <v>50000</v>
+      </c>
+      <c r="H13" t="str">
+        <v>CLAUSE DEAL · joined as Starter</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>1783473413103</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" t="str">
+        <v>FA SIGNING</v>
+      </c>
+      <c r="D14" t="str">
+        <v>taco</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Free Agency</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="G14">
         <v>0</v>
       </c>
-      <c r="H12" t="str">
+      <c r="H14" t="str">
+        <v>joined as Starter</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>1783473388452</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" t="str">
+        <v>FA SIGNING</v>
+      </c>
+      <c r="D15" t="str">
+        <v>fer</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Free Agency</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" t="str">
         <v>joined as Starter</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>playerName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>buyer</v>
+      </c>
+      <c r="D1" t="str">
+        <v>seller</v>
+      </c>
+      <c r="E1" t="str">
+        <v>amount</v>
+      </c>
+      <c r="F1" t="str">
+        <v>status</v>
+      </c>
+      <c r="G1" t="str">
+        <v>month</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1785396010605</v>
+      </c>
+      <c r="B2" t="str">
+        <v>boltz</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Lux Tenebris</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FREE AGENCY</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>✅ FA SIGNING</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>